<commit_message>
Commit before merging main to incorporate monteprep code
</commit_message>
<xml_diff>
--- a/results_analysis.xlsx
+++ b/results_analysis.xlsx
@@ -22,13 +22,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +50,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,11 +430,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -431,37 +443,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Planning</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Length</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Cases Evaluated</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Avg Cost ($)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Avg Latency (s)</t>
         </is>
@@ -774,10 +786,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E12" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F12" t="n">
         <v>0.051184</v>
@@ -803,10 +815,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>62</v>
+        <v>97</v>
       </c>
       <c r="E13" t="n">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="F13" t="n">
         <v>0.049883</v>
@@ -1074,6 +1086,93 @@
       </c>
       <c r="G22" t="n">
         <v>165.75</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Operator-driven</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>100</v>
+      </c>
+      <c r="E23" t="n">
+        <v>80</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.010243</v>
+      </c>
+      <c r="G23" t="n">
+        <v>62.2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Operator-driven</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>81</v>
+      </c>
+      <c r="E24" t="n">
+        <v>32</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.030905</v>
+      </c>
+      <c r="G24" t="n">
+        <v>181.93</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Operator-driven</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>L9</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>84</v>
+      </c>
+      <c r="E25" t="n">
+        <v>61</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.025543</v>
+      </c>
+      <c r="G25" t="n">
+        <v>113.69</v>
       </c>
     </row>
   </sheetData>
@@ -1087,7 +1186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H102"/>
+  <dimension ref="A1:I102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1098,56 +1197,63 @@
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="29" customWidth="1" min="8" max="8"/>
+    <col width="43" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Case ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Operator-driven
 CoT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Operator-driven
 Critique</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Operator-driven
 Iterative</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Operator-driven
 MCTS</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Pipeline-driven
 CoT</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Pipeline-driven
 Critique</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Pipeline-driven
 Iterative</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Operator-driven
+Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1176,6 +1282,9 @@
       <c r="H2" t="b">
         <v>1</v>
       </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1204,6 +1313,9 @@
       <c r="H3" t="b">
         <v>1</v>
       </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1232,6 +1344,9 @@
       <c r="H4" t="b">
         <v>1</v>
       </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1260,6 +1375,9 @@
       <c r="H5" t="b">
         <v>1</v>
       </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1288,6 +1406,9 @@
       <c r="H6" t="b">
         <v>1</v>
       </c>
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1316,6 +1437,9 @@
       <c r="H7" t="b">
         <v>1</v>
       </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1344,6 +1468,9 @@
       <c r="H8" t="b">
         <v>1</v>
       </c>
+      <c r="I8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1372,6 +1499,9 @@
       <c r="H9" t="b">
         <v>1</v>
       </c>
+      <c r="I9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1400,6 +1530,9 @@
       <c r="H10" t="b">
         <v>1</v>
       </c>
+      <c r="I10" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1428,6 +1561,9 @@
       <c r="H11" t="b">
         <v>0</v>
       </c>
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1456,6 +1592,9 @@
       <c r="H12" t="b">
         <v>1</v>
       </c>
+      <c r="I12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1484,6 +1623,9 @@
       <c r="H13" t="b">
         <v>1</v>
       </c>
+      <c r="I13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1512,6 +1654,9 @@
       <c r="H14" t="b">
         <v>1</v>
       </c>
+      <c r="I14" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1540,6 +1685,9 @@
       <c r="H15" t="b">
         <v>0</v>
       </c>
+      <c r="I15" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1568,6 +1716,9 @@
       <c r="H16" t="b">
         <v>1</v>
       </c>
+      <c r="I16" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1596,6 +1747,9 @@
       <c r="H17" t="b">
         <v>1</v>
       </c>
+      <c r="I17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1624,6 +1778,9 @@
       <c r="H18" t="b">
         <v>0</v>
       </c>
+      <c r="I18" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1652,6 +1809,9 @@
       <c r="H19" t="b">
         <v>1</v>
       </c>
+      <c r="I19" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1680,6 +1840,9 @@
       <c r="H20" t="b">
         <v>0</v>
       </c>
+      <c r="I20" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1708,6 +1871,9 @@
       <c r="H21" t="b">
         <v>1</v>
       </c>
+      <c r="I21" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1736,6 +1902,9 @@
       <c r="H22" t="b">
         <v>0</v>
       </c>
+      <c r="I22" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1764,6 +1933,9 @@
       <c r="H23" t="b">
         <v>0</v>
       </c>
+      <c r="I23" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1792,6 +1964,9 @@
       <c r="H24" t="b">
         <v>0</v>
       </c>
+      <c r="I24" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1820,6 +1995,9 @@
       <c r="H25" t="b">
         <v>0</v>
       </c>
+      <c r="I25" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1848,6 +2026,9 @@
       <c r="H26" t="b">
         <v>0</v>
       </c>
+      <c r="I26" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1876,6 +2057,9 @@
       <c r="H27" t="b">
         <v>1</v>
       </c>
+      <c r="I27" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1904,6 +2088,9 @@
       <c r="H28" t="b">
         <v>1</v>
       </c>
+      <c r="I28" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1932,6 +2119,9 @@
       <c r="H29" t="b">
         <v>0</v>
       </c>
+      <c r="I29" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1960,6 +2150,9 @@
       <c r="H30" t="b">
         <v>1</v>
       </c>
+      <c r="I30" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1988,6 +2181,9 @@
       <c r="H31" t="b">
         <v>1</v>
       </c>
+      <c r="I31" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2016,6 +2212,9 @@
       <c r="H32" t="b">
         <v>1</v>
       </c>
+      <c r="I32" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2044,6 +2243,9 @@
       <c r="H33" t="b">
         <v>1</v>
       </c>
+      <c r="I33" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2072,6 +2274,9 @@
       <c r="H34" t="b">
         <v>1</v>
       </c>
+      <c r="I34" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2100,6 +2305,9 @@
       <c r="H35" t="b">
         <v>1</v>
       </c>
+      <c r="I35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2128,6 +2336,9 @@
       <c r="H36" t="b">
         <v>1</v>
       </c>
+      <c r="I36" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2156,6 +2367,9 @@
       <c r="H37" t="b">
         <v>1</v>
       </c>
+      <c r="I37" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2184,6 +2398,9 @@
       <c r="H38" t="b">
         <v>1</v>
       </c>
+      <c r="I38" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2212,6 +2429,9 @@
       <c r="H39" t="b">
         <v>0</v>
       </c>
+      <c r="I39" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2240,6 +2460,9 @@
       <c r="H40" t="b">
         <v>1</v>
       </c>
+      <c r="I40" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2268,6 +2491,9 @@
       <c r="H41" t="b">
         <v>1</v>
       </c>
+      <c r="I41" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2296,6 +2522,9 @@
       <c r="H42" t="b">
         <v>0</v>
       </c>
+      <c r="I42" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2324,6 +2553,9 @@
       <c r="H43" t="b">
         <v>0</v>
       </c>
+      <c r="I43" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2352,6 +2584,9 @@
       <c r="H44" t="b">
         <v>1</v>
       </c>
+      <c r="I44" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2380,6 +2615,9 @@
       <c r="H45" t="b">
         <v>0</v>
       </c>
+      <c r="I45" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2408,6 +2646,9 @@
       <c r="H46" t="b">
         <v>0</v>
       </c>
+      <c r="I46" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2436,6 +2677,9 @@
       <c r="H47" t="b">
         <v>1</v>
       </c>
+      <c r="I47" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2464,6 +2708,9 @@
       <c r="H48" t="b">
         <v>0</v>
       </c>
+      <c r="I48" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2492,6 +2739,9 @@
       <c r="H49" t="b">
         <v>1</v>
       </c>
+      <c r="I49" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2520,6 +2770,9 @@
       <c r="H50" t="b">
         <v>0</v>
       </c>
+      <c r="I50" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2548,6 +2801,9 @@
       <c r="H51" t="b">
         <v>1</v>
       </c>
+      <c r="I51" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2576,6 +2832,9 @@
       <c r="H52" t="b">
         <v>1</v>
       </c>
+      <c r="I52" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2604,6 +2863,9 @@
       <c r="H53" t="b">
         <v>1</v>
       </c>
+      <c r="I53" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2632,6 +2894,9 @@
       <c r="H54" t="b">
         <v>0</v>
       </c>
+      <c r="I54" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2660,6 +2925,9 @@
       <c r="H55" t="b">
         <v>0</v>
       </c>
+      <c r="I55" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2688,6 +2956,9 @@
       <c r="H56" t="b">
         <v>0</v>
       </c>
+      <c r="I56" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2716,6 +2987,9 @@
       <c r="H57" t="b">
         <v>1</v>
       </c>
+      <c r="I57" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2744,6 +3018,9 @@
       <c r="H58" t="b">
         <v>1</v>
       </c>
+      <c r="I58" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2772,6 +3049,9 @@
       <c r="H59" t="b">
         <v>1</v>
       </c>
+      <c r="I59" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2800,6 +3080,9 @@
       <c r="H60" t="b">
         <v>1</v>
       </c>
+      <c r="I60" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2828,6 +3111,9 @@
       <c r="H61" t="b">
         <v>1</v>
       </c>
+      <c r="I61" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2856,6 +3142,9 @@
       <c r="H62" t="b">
         <v>0</v>
       </c>
+      <c r="I62" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2884,6 +3173,9 @@
       <c r="H63" t="b">
         <v>0</v>
       </c>
+      <c r="I63" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2912,6 +3204,9 @@
       <c r="H64" t="b">
         <v>0</v>
       </c>
+      <c r="I64" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2940,6 +3235,9 @@
       <c r="H65" t="b">
         <v>1</v>
       </c>
+      <c r="I65" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2968,6 +3266,9 @@
       <c r="H66" t="b">
         <v>1</v>
       </c>
+      <c r="I66" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2996,6 +3297,9 @@
       <c r="H67" t="b">
         <v>0</v>
       </c>
+      <c r="I67" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3024,6 +3328,9 @@
       <c r="H68" t="b">
         <v>1</v>
       </c>
+      <c r="I68" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3052,6 +3359,9 @@
       <c r="H69" t="b">
         <v>1</v>
       </c>
+      <c r="I69" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3080,6 +3390,9 @@
       <c r="H70" t="b">
         <v>1</v>
       </c>
+      <c r="I70" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3108,6 +3421,9 @@
       <c r="H71" t="b">
         <v>1</v>
       </c>
+      <c r="I71" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3136,6 +3452,9 @@
       <c r="H72" t="b">
         <v>1</v>
       </c>
+      <c r="I72" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3164,6 +3483,9 @@
       <c r="H73" t="b">
         <v>1</v>
       </c>
+      <c r="I73" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3192,6 +3514,9 @@
       <c r="H74" t="b">
         <v>0</v>
       </c>
+      <c r="I74" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3220,6 +3545,9 @@
       <c r="H75" t="b">
         <v>1</v>
       </c>
+      <c r="I75" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3248,6 +3576,9 @@
       <c r="H76" t="b">
         <v>1</v>
       </c>
+      <c r="I76" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3276,6 +3607,9 @@
       <c r="H77" t="b">
         <v>0</v>
       </c>
+      <c r="I77" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3304,6 +3638,9 @@
       <c r="H78" t="b">
         <v>1</v>
       </c>
+      <c r="I78" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3332,6 +3669,9 @@
       <c r="H79" t="b">
         <v>0</v>
       </c>
+      <c r="I79" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3360,6 +3700,9 @@
       <c r="H80" t="b">
         <v>0</v>
       </c>
+      <c r="I80" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3388,6 +3731,9 @@
       <c r="H81" t="b">
         <v>1</v>
       </c>
+      <c r="I81" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3416,6 +3762,9 @@
       <c r="H82" t="b">
         <v>1</v>
       </c>
+      <c r="I82" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3444,6 +3793,9 @@
       <c r="H83" t="b">
         <v>0</v>
       </c>
+      <c r="I83" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3472,6 +3824,9 @@
       <c r="H84" t="b">
         <v>0</v>
       </c>
+      <c r="I84" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3500,6 +3855,9 @@
       <c r="H85" t="b">
         <v>1</v>
       </c>
+      <c r="I85" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3528,6 +3886,9 @@
       <c r="H86" t="b">
         <v>1</v>
       </c>
+      <c r="I86" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3556,6 +3917,9 @@
       <c r="H87" t="b">
         <v>1</v>
       </c>
+      <c r="I87" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3584,6 +3948,9 @@
       <c r="H88" t="b">
         <v>0</v>
       </c>
+      <c r="I88" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3612,6 +3979,9 @@
       <c r="H89" t="b">
         <v>0</v>
       </c>
+      <c r="I89" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3640,6 +4010,9 @@
       <c r="H90" t="b">
         <v>1</v>
       </c>
+      <c r="I90" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3668,6 +4041,9 @@
       <c r="H91" t="b">
         <v>0</v>
       </c>
+      <c r="I91" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3696,6 +4072,9 @@
       <c r="H92" t="b">
         <v>0</v>
       </c>
+      <c r="I92" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3724,6 +4103,9 @@
       <c r="H93" t="b">
         <v>0</v>
       </c>
+      <c r="I93" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3752,6 +4134,9 @@
       <c r="H94" t="b">
         <v>0</v>
       </c>
+      <c r="I94" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3780,6 +4165,9 @@
       <c r="H95" t="b">
         <v>0</v>
       </c>
+      <c r="I95" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3808,6 +4196,9 @@
       <c r="H96" t="b">
         <v>0</v>
       </c>
+      <c r="I96" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3836,6 +4227,9 @@
       <c r="H97" t="b">
         <v>0</v>
       </c>
+      <c r="I97" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3864,6 +4258,9 @@
       <c r="H98" t="b">
         <v>0</v>
       </c>
+      <c r="I98" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3892,6 +4289,9 @@
       <c r="H99" t="b">
         <v>0</v>
       </c>
+      <c r="I99" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3920,6 +4320,9 @@
       <c r="H100" t="b">
         <v>0</v>
       </c>
+      <c r="I100" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3948,6 +4351,9 @@
       <c r="H101" t="b">
         <v>0</v>
       </c>
+      <c r="I101" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3982,6 +4388,11 @@
         <v>0</v>
       </c>
       <c r="H102" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -3998,7 +4409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:I86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4009,56 +4420,63 @@
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="29" customWidth="1" min="8" max="8"/>
+    <col width="43" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Case ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Operator-driven
 CoT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Operator-driven
 Critique</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Operator-driven
 Iterative</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Operator-driven
 MCTS</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Pipeline-driven
 CoT</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Pipeline-driven
 Critique</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Pipeline-driven
 Iterative</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Operator-driven
+Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4087,6 +4505,9 @@
       <c r="H2" t="b">
         <v>0</v>
       </c>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4115,6 +4536,9 @@
       <c r="H3" t="b">
         <v>0</v>
       </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4143,6 +4567,9 @@
       <c r="H4" t="b">
         <v>0</v>
       </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4171,6 +4598,9 @@
       <c r="H5" t="b">
         <v>0</v>
       </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4199,6 +4629,9 @@
       <c r="H6" t="b">
         <v>0</v>
       </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4227,6 +4660,9 @@
       <c r="H7" t="b">
         <v>0</v>
       </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4255,6 +4691,9 @@
       <c r="H8" t="b">
         <v>0</v>
       </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4283,6 +4722,9 @@
       <c r="H9" t="b">
         <v>0</v>
       </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4311,6 +4753,9 @@
       <c r="H10" t="b">
         <v>0</v>
       </c>
+      <c r="I10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4339,6 +4784,9 @@
       <c r="H11" t="b">
         <v>0</v>
       </c>
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4367,6 +4815,9 @@
       <c r="H12" t="b">
         <v>0</v>
       </c>
+      <c r="I12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4395,6 +4846,9 @@
       <c r="H13" t="b">
         <v>0</v>
       </c>
+      <c r="I13" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4412,7 +4866,7 @@
         <v>0</v>
       </c>
       <c r="E14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" t="b">
         <v>0</v>
@@ -4421,6 +4875,9 @@
         <v>0</v>
       </c>
       <c r="H14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4451,6 +4908,9 @@
       <c r="H15" t="b">
         <v>0</v>
       </c>
+      <c r="I15" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4479,6 +4939,9 @@
       <c r="H16" t="b">
         <v>0</v>
       </c>
+      <c r="I16" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4507,6 +4970,9 @@
       <c r="H17" t="b">
         <v>1</v>
       </c>
+      <c r="I17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4535,6 +5001,9 @@
       <c r="H18" t="b">
         <v>0</v>
       </c>
+      <c r="I18" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4563,6 +5032,9 @@
       <c r="H19" t="b">
         <v>0</v>
       </c>
+      <c r="I19" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4591,6 +5063,9 @@
       <c r="H20" t="b">
         <v>1</v>
       </c>
+      <c r="I20" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4619,6 +5094,9 @@
       <c r="H21" t="b">
         <v>1</v>
       </c>
+      <c r="I21" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4647,6 +5125,9 @@
       <c r="H22" t="b">
         <v>0</v>
       </c>
+      <c r="I22" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4675,6 +5156,9 @@
       <c r="H23" t="b">
         <v>0</v>
       </c>
+      <c r="I23" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4703,6 +5187,9 @@
       <c r="H24" t="b">
         <v>1</v>
       </c>
+      <c r="I24" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4720,7 +5207,7 @@
         <v>1</v>
       </c>
       <c r="E25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" t="b">
         <v>0</v>
@@ -4729,6 +5216,9 @@
         <v>0</v>
       </c>
       <c r="H25" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4748,7 +5238,7 @@
         <v>0</v>
       </c>
       <c r="E26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" t="b">
         <v>0</v>
@@ -4758,6 +5248,9 @@
       </c>
       <c r="H26" t="b">
         <v>0</v>
+      </c>
+      <c r="I26" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -4776,7 +5269,7 @@
         <v>1</v>
       </c>
       <c r="E27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F27" t="b">
         <v>0</v>
@@ -4786,6 +5279,9 @@
       </c>
       <c r="H27" t="b">
         <v>0</v>
+      </c>
+      <c r="I27" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -4804,7 +5300,7 @@
         <v>0</v>
       </c>
       <c r="E28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" t="b">
         <v>1</v>
@@ -4814,6 +5310,9 @@
       </c>
       <c r="H28" t="b">
         <v>0</v>
+      </c>
+      <c r="I28" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -4843,6 +5342,9 @@
       <c r="H29" t="b">
         <v>0</v>
       </c>
+      <c r="I29" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4871,6 +5373,9 @@
       <c r="H30" t="b">
         <v>0</v>
       </c>
+      <c r="I30" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4899,6 +5404,9 @@
       <c r="H31" t="b">
         <v>0</v>
       </c>
+      <c r="I31" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4927,6 +5435,9 @@
       <c r="H32" t="b">
         <v>0</v>
       </c>
+      <c r="I32" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4955,6 +5466,9 @@
       <c r="H33" t="b">
         <v>0</v>
       </c>
+      <c r="I33" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4983,6 +5497,9 @@
       <c r="H34" t="b">
         <v>0</v>
       </c>
+      <c r="I34" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5011,6 +5528,9 @@
       <c r="H35" t="b">
         <v>0</v>
       </c>
+      <c r="I35" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5039,6 +5559,9 @@
       <c r="H36" t="b">
         <v>0</v>
       </c>
+      <c r="I36" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5067,6 +5590,9 @@
       <c r="H37" t="b">
         <v>0</v>
       </c>
+      <c r="I37" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5095,6 +5621,9 @@
       <c r="H38" t="b">
         <v>0</v>
       </c>
+      <c r="I38" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5123,6 +5652,9 @@
       <c r="H39" t="b">
         <v>0</v>
       </c>
+      <c r="I39" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5151,6 +5683,9 @@
       <c r="H40" t="b">
         <v>0</v>
       </c>
+      <c r="I40" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5179,6 +5714,9 @@
       <c r="H41" t="b">
         <v>0</v>
       </c>
+      <c r="I41" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5207,6 +5745,9 @@
       <c r="H42" t="b">
         <v>1</v>
       </c>
+      <c r="I42" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5235,6 +5776,9 @@
       <c r="H43" t="b">
         <v>0</v>
       </c>
+      <c r="I43" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5263,6 +5807,9 @@
       <c r="H44" t="b">
         <v>0</v>
       </c>
+      <c r="I44" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5280,7 +5827,7 @@
         <v>0</v>
       </c>
       <c r="E45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F45" t="b">
         <v>0</v>
@@ -5289,6 +5836,9 @@
         <v>0</v>
       </c>
       <c r="H45" t="b">
+        <v>0</v>
+      </c>
+      <c r="I45" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5319,6 +5869,9 @@
       <c r="H46" t="b">
         <v>0</v>
       </c>
+      <c r="I46" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5347,6 +5900,9 @@
       <c r="H47" t="b">
         <v>0</v>
       </c>
+      <c r="I47" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5375,6 +5931,9 @@
       <c r="H48" t="b">
         <v>0</v>
       </c>
+      <c r="I48" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5411,6 +5970,11 @@
       <c r="H49" t="b">
         <v>0</v>
       </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5447,6 +6011,11 @@
       <c r="H50" t="b">
         <v>0</v>
       </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5483,6 +6052,11 @@
       <c r="H51" t="b">
         <v>0</v>
       </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5500,7 +6074,7 @@
         <v>0</v>
       </c>
       <c r="E52" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F52" t="b">
         <v>1</v>
@@ -5509,6 +6083,9 @@
         <v>1</v>
       </c>
       <c r="H52" t="b">
+        <v>1</v>
+      </c>
+      <c r="I52" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5539,6 +6116,9 @@
       <c r="H53" t="b">
         <v>1</v>
       </c>
+      <c r="I53" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5567,6 +6147,9 @@
       <c r="H54" t="b">
         <v>0</v>
       </c>
+      <c r="I54" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5595,6 +6178,9 @@
       <c r="H55" t="b">
         <v>0</v>
       </c>
+      <c r="I55" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5623,6 +6209,9 @@
       <c r="H56" t="b">
         <v>1</v>
       </c>
+      <c r="I56" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5651,6 +6240,9 @@
       <c r="H57" t="b">
         <v>0</v>
       </c>
+      <c r="I57" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5679,6 +6271,9 @@
       <c r="H58" t="b">
         <v>0</v>
       </c>
+      <c r="I58" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5696,7 +6291,7 @@
         <v>1</v>
       </c>
       <c r="E59" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F59" t="b">
         <v>0</v>
@@ -5705,6 +6300,9 @@
         <v>1</v>
       </c>
       <c r="H59" t="b">
+        <v>0</v>
+      </c>
+      <c r="I59" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5735,6 +6333,9 @@
       <c r="H60" t="b">
         <v>0</v>
       </c>
+      <c r="I60" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5763,6 +6364,9 @@
       <c r="H61" t="b">
         <v>0</v>
       </c>
+      <c r="I61" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5780,7 +6384,7 @@
         <v>1</v>
       </c>
       <c r="E62" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F62" t="b">
         <v>1</v>
@@ -5789,6 +6393,9 @@
         <v>1</v>
       </c>
       <c r="H62" t="b">
+        <v>1</v>
+      </c>
+      <c r="I62" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5819,6 +6426,9 @@
       <c r="H63" t="b">
         <v>0</v>
       </c>
+      <c r="I63" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5847,6 +6457,9 @@
       <c r="H64" t="b">
         <v>0</v>
       </c>
+      <c r="I64" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5864,7 +6477,7 @@
         <v>0</v>
       </c>
       <c r="E65" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F65" t="b">
         <v>0</v>
@@ -5874,6 +6487,9 @@
       </c>
       <c r="H65" t="b">
         <v>0</v>
+      </c>
+      <c r="I65" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -5903,6 +6519,9 @@
       <c r="H66" t="b">
         <v>1</v>
       </c>
+      <c r="I66" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5920,7 +6539,7 @@
         <v>0</v>
       </c>
       <c r="E67" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F67" t="b">
         <v>0</v>
@@ -5930,6 +6549,9 @@
       </c>
       <c r="H67" t="b">
         <v>0</v>
+      </c>
+      <c r="I67" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="68">
@@ -5959,6 +6581,9 @@
       <c r="H68" t="b">
         <v>0</v>
       </c>
+      <c r="I68" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5976,7 +6601,7 @@
         <v>1</v>
       </c>
       <c r="E69" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F69" t="b">
         <v>0</v>
@@ -5986,6 +6611,9 @@
       </c>
       <c r="H69" t="b">
         <v>0</v>
+      </c>
+      <c r="I69" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -6015,6 +6643,9 @@
       <c r="H70" t="b">
         <v>1</v>
       </c>
+      <c r="I70" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6032,7 +6663,7 @@
         <v>0</v>
       </c>
       <c r="E71" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F71" t="b">
         <v>0</v>
@@ -6042,6 +6673,9 @@
       </c>
       <c r="H71" t="b">
         <v>0</v>
+      </c>
+      <c r="I71" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -6060,7 +6694,7 @@
         <v>1</v>
       </c>
       <c r="E72" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F72" t="b">
         <v>0</v>
@@ -6070,6 +6704,9 @@
       </c>
       <c r="H72" t="b">
         <v>0</v>
+      </c>
+      <c r="I72" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -6099,6 +6736,9 @@
       <c r="H73" t="b">
         <v>0</v>
       </c>
+      <c r="I73" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6135,6 +6775,11 @@
       <c r="H74" t="b">
         <v>0</v>
       </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6152,7 +6797,7 @@
         <v>1</v>
       </c>
       <c r="E75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F75" t="b">
         <v>1</v>
@@ -6161,6 +6806,9 @@
         <v>1</v>
       </c>
       <c r="H75" t="b">
+        <v>1</v>
+      </c>
+      <c r="I75" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6180,7 +6828,7 @@
         <v>1</v>
       </c>
       <c r="E76" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F76" t="b">
         <v>1</v>
@@ -6189,6 +6837,9 @@
         <v>1</v>
       </c>
       <c r="H76" t="b">
+        <v>1</v>
+      </c>
+      <c r="I76" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6208,7 +6859,7 @@
         <v>0</v>
       </c>
       <c r="E77" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F77" t="b">
         <v>0</v>
@@ -6218,6 +6869,9 @@
       </c>
       <c r="H77" t="b">
         <v>0</v>
+      </c>
+      <c r="I77" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -6236,7 +6890,7 @@
         <v>0</v>
       </c>
       <c r="E78" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F78" t="b">
         <v>0</v>
@@ -6246,6 +6900,9 @@
       </c>
       <c r="H78" t="b">
         <v>0</v>
+      </c>
+      <c r="I78" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="79">
@@ -6275,6 +6932,9 @@
       <c r="H79" t="b">
         <v>0</v>
       </c>
+      <c r="I79" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6303,6 +6963,9 @@
       <c r="H80" t="b">
         <v>0</v>
       </c>
+      <c r="I80" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6331,6 +6994,9 @@
       <c r="H81" t="b">
         <v>0</v>
       </c>
+      <c r="I81" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6359,6 +7025,9 @@
       <c r="H82" t="b">
         <v>0</v>
       </c>
+      <c r="I82" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6387,6 +7056,9 @@
       <c r="H83" t="b">
         <v>0</v>
       </c>
+      <c r="I83" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6415,6 +7087,9 @@
       <c r="H84" t="b">
         <v>0</v>
       </c>
+      <c r="I84" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6443,6 +7118,9 @@
       <c r="H85" t="b">
         <v>0</v>
       </c>
+      <c r="I85" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6469,6 +7147,9 @@
         <v>0</v>
       </c>
       <c r="H86" t="b">
+        <v>0</v>
+      </c>
+      <c r="I86" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6483,7 +7164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H102"/>
+  <dimension ref="A1:I102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6494,56 +7175,63 @@
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="29" customWidth="1" min="8" max="8"/>
+    <col width="43" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Case ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Operator-driven
 CoT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Operator-driven
 Critique</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Operator-driven
 Iterative</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Operator-driven
 MCTS</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Pipeline-driven
 CoT</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Pipeline-driven
 Critique</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Pipeline-driven
 Iterative</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Operator-driven
+Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -6572,6 +7260,9 @@
       <c r="H2" t="b">
         <v>0</v>
       </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6600,6 +7291,9 @@
       <c r="H3" t="b">
         <v>0</v>
       </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6628,6 +7322,9 @@
       <c r="H4" t="b">
         <v>0</v>
       </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6656,6 +7353,9 @@
       <c r="H5" t="b">
         <v>0</v>
       </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6684,6 +7384,9 @@
       <c r="H6" t="b">
         <v>0</v>
       </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6712,6 +7415,9 @@
       <c r="H7" t="b">
         <v>1</v>
       </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6740,6 +7446,9 @@
       <c r="H8" t="b">
         <v>0</v>
       </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6768,6 +7477,9 @@
       <c r="H9" t="b">
         <v>1</v>
       </c>
+      <c r="I9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6796,6 +7508,9 @@
       <c r="H10" t="b">
         <v>1</v>
       </c>
+      <c r="I10" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6824,6 +7539,9 @@
       <c r="H11" t="b">
         <v>1</v>
       </c>
+      <c r="I11" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6852,6 +7570,9 @@
       <c r="H12" t="b">
         <v>1</v>
       </c>
+      <c r="I12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6880,6 +7601,9 @@
       <c r="H13" t="b">
         <v>1</v>
       </c>
+      <c r="I13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6908,6 +7632,9 @@
       <c r="H14" t="b">
         <v>1</v>
       </c>
+      <c r="I14" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6944,6 +7671,11 @@
       <c r="H15" t="b">
         <v>0</v>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6972,6 +7704,9 @@
       <c r="H16" t="b">
         <v>1</v>
       </c>
+      <c r="I16" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7000,6 +7735,9 @@
       <c r="H17" t="b">
         <v>0</v>
       </c>
+      <c r="I17" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7028,6 +7766,9 @@
       <c r="H18" t="b">
         <v>1</v>
       </c>
+      <c r="I18" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7056,6 +7797,9 @@
       <c r="H19" t="b">
         <v>1</v>
       </c>
+      <c r="I19" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7084,6 +7828,11 @@
       <c r="H20" t="b">
         <v>0</v>
       </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7112,6 +7861,9 @@
       <c r="H21" t="b">
         <v>0</v>
       </c>
+      <c r="I21" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7140,6 +7892,11 @@
       <c r="H22" t="b">
         <v>0</v>
       </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7168,6 +7925,11 @@
       <c r="H23" t="b">
         <v>0</v>
       </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7185,7 +7947,7 @@
         <v>0</v>
       </c>
       <c r="E24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F24" t="b">
         <v>0</v>
@@ -7195,6 +7957,9 @@
       </c>
       <c r="H24" t="b">
         <v>0</v>
+      </c>
+      <c r="I24" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -7213,7 +7978,7 @@
         <v>0</v>
       </c>
       <c r="E25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" t="b">
         <v>0</v>
@@ -7223,6 +7988,9 @@
       </c>
       <c r="H25" t="b">
         <v>0</v>
+      </c>
+      <c r="I25" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -7252,6 +8020,9 @@
       <c r="H26" t="b">
         <v>0</v>
       </c>
+      <c r="I26" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7280,6 +8051,9 @@
       <c r="H27" t="b">
         <v>0</v>
       </c>
+      <c r="I27" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7308,6 +8082,9 @@
       <c r="H28" t="b">
         <v>0</v>
       </c>
+      <c r="I28" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7336,6 +8113,9 @@
       <c r="H29" t="b">
         <v>0</v>
       </c>
+      <c r="I29" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7353,7 +8133,7 @@
         <v>0</v>
       </c>
       <c r="E30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" t="b">
         <v>0</v>
@@ -7362,6 +8142,9 @@
         <v>0</v>
       </c>
       <c r="H30" t="b">
+        <v>0</v>
+      </c>
+      <c r="I30" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7392,6 +8175,9 @@
       <c r="H31" t="b">
         <v>1</v>
       </c>
+      <c r="I31" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7420,6 +8206,9 @@
       <c r="H32" t="b">
         <v>1</v>
       </c>
+      <c r="I32" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7448,6 +8237,9 @@
       <c r="H33" t="b">
         <v>0</v>
       </c>
+      <c r="I33" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7476,6 +8268,9 @@
       <c r="H34" t="b">
         <v>1</v>
       </c>
+      <c r="I34" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7493,7 +8288,7 @@
         <v>0</v>
       </c>
       <c r="E35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35" t="b">
         <v>0</v>
@@ -7502,6 +8297,9 @@
         <v>0</v>
       </c>
       <c r="H35" t="b">
+        <v>0</v>
+      </c>
+      <c r="I35" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7521,7 +8319,7 @@
         <v>0</v>
       </c>
       <c r="E36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F36" t="b">
         <v>0</v>
@@ -7530,6 +8328,9 @@
         <v>0</v>
       </c>
       <c r="H36" t="b">
+        <v>1</v>
+      </c>
+      <c r="I36" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7549,7 +8350,7 @@
         <v>1</v>
       </c>
       <c r="E37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F37" t="b">
         <v>0</v>
@@ -7559,6 +8360,9 @@
       </c>
       <c r="H37" t="b">
         <v>1</v>
+      </c>
+      <c r="I37" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -7596,6 +8400,11 @@
       <c r="H38" t="b">
         <v>0</v>
       </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -7624,6 +8433,9 @@
       <c r="H39" t="b">
         <v>0</v>
       </c>
+      <c r="I39" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7652,6 +8464,9 @@
       <c r="H40" t="b">
         <v>0</v>
       </c>
+      <c r="I40" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -7680,6 +8495,9 @@
       <c r="H41" t="b">
         <v>0</v>
       </c>
+      <c r="I41" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -7708,6 +8526,9 @@
       <c r="H42" t="b">
         <v>0</v>
       </c>
+      <c r="I42" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -7744,6 +8565,11 @@
       <c r="H43" t="b">
         <v>1</v>
       </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -7780,6 +8606,11 @@
       <c r="H44" t="b">
         <v>0</v>
       </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -7816,6 +8647,11 @@
       <c r="H45" t="b">
         <v>0</v>
       </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -7852,6 +8688,11 @@
       <c r="H46" t="b">
         <v>1</v>
       </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -7888,6 +8729,11 @@
       <c r="H47" t="b">
         <v>0</v>
       </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -7916,6 +8762,9 @@
       <c r="H48" t="b">
         <v>0</v>
       </c>
+      <c r="I48" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -7944,6 +8793,9 @@
       <c r="H49" t="b">
         <v>0</v>
       </c>
+      <c r="I49" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -7972,6 +8824,9 @@
       <c r="H50" t="b">
         <v>1</v>
       </c>
+      <c r="I50" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8000,6 +8855,9 @@
       <c r="H51" t="b">
         <v>0</v>
       </c>
+      <c r="I51" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -8028,6 +8886,9 @@
       <c r="H52" t="b">
         <v>1</v>
       </c>
+      <c r="I52" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -8056,6 +8917,9 @@
       <c r="H53" t="b">
         <v>0</v>
       </c>
+      <c r="I53" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -8084,6 +8948,9 @@
       <c r="H54" t="b">
         <v>0</v>
       </c>
+      <c r="I54" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -8112,6 +8979,9 @@
       <c r="H55" t="b">
         <v>0</v>
       </c>
+      <c r="I55" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -8140,6 +9010,9 @@
       <c r="H56" t="b">
         <v>1</v>
       </c>
+      <c r="I56" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -8168,6 +9041,9 @@
       <c r="H57" t="b">
         <v>1</v>
       </c>
+      <c r="I57" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -8196,6 +9072,9 @@
       <c r="H58" t="b">
         <v>0</v>
       </c>
+      <c r="I58" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -8224,6 +9103,9 @@
       <c r="H59" t="b">
         <v>0</v>
       </c>
+      <c r="I59" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -8252,6 +9134,9 @@
       <c r="H60" t="b">
         <v>1</v>
       </c>
+      <c r="I60" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8280,6 +9165,9 @@
       <c r="H61" t="b">
         <v>0</v>
       </c>
+      <c r="I61" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -8308,6 +9196,9 @@
       <c r="H62" t="b">
         <v>1</v>
       </c>
+      <c r="I62" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -8336,6 +9227,9 @@
       <c r="H63" t="b">
         <v>1</v>
       </c>
+      <c r="I63" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -8372,6 +9266,11 @@
       <c r="H64" t="b">
         <v>0</v>
       </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8400,6 +9299,9 @@
       <c r="H65" t="b">
         <v>1</v>
       </c>
+      <c r="I65" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8428,6 +9330,9 @@
       <c r="H66" t="b">
         <v>1</v>
       </c>
+      <c r="I66" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -8445,7 +9350,7 @@
         <v>1</v>
       </c>
       <c r="E67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F67" t="b">
         <v>0</v>
@@ -8454,6 +9359,9 @@
         <v>1</v>
       </c>
       <c r="H67" t="b">
+        <v>1</v>
+      </c>
+      <c r="I67" t="b">
         <v>1</v>
       </c>
     </row>
@@ -8484,6 +9392,9 @@
       <c r="H68" t="b">
         <v>1</v>
       </c>
+      <c r="I68" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -8512,6 +9423,9 @@
       <c r="H69" t="b">
         <v>0</v>
       </c>
+      <c r="I69" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -8540,6 +9454,9 @@
       <c r="H70" t="b">
         <v>0</v>
       </c>
+      <c r="I70" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8568,6 +9485,9 @@
       <c r="H71" t="b">
         <v>0</v>
       </c>
+      <c r="I71" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -8596,6 +9516,9 @@
       <c r="H72" t="b">
         <v>0</v>
       </c>
+      <c r="I72" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8626,6 +9549,11 @@
       <c r="H73" t="b">
         <v>0</v>
       </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8660,6 +9588,11 @@
       <c r="H74" t="b">
         <v>0</v>
       </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8690,6 +9623,9 @@
       <c r="H75" t="b">
         <v>0</v>
       </c>
+      <c r="I75" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -8720,6 +9656,11 @@
       <c r="H76" t="b">
         <v>0</v>
       </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -8748,6 +9689,9 @@
       <c r="H77" t="b">
         <v>1</v>
       </c>
+      <c r="I77" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -8776,6 +9720,9 @@
       <c r="H78" t="b">
         <v>1</v>
       </c>
+      <c r="I78" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8804,6 +9751,9 @@
       <c r="H79" t="b">
         <v>1</v>
       </c>
+      <c r="I79" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -8840,6 +9790,11 @@
       <c r="H80" t="b">
         <v>1</v>
       </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -8876,6 +9831,11 @@
       <c r="H81" t="b">
         <v>1</v>
       </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -8904,6 +9864,9 @@
       <c r="H82" t="b">
         <v>1</v>
       </c>
+      <c r="I82" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -8932,6 +9895,9 @@
       <c r="H83" t="b">
         <v>1</v>
       </c>
+      <c r="I83" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -8960,6 +9926,9 @@
       <c r="H84" t="b">
         <v>1</v>
       </c>
+      <c r="I84" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -8988,6 +9957,9 @@
       <c r="H85" t="b">
         <v>1</v>
       </c>
+      <c r="I85" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -9016,6 +9988,9 @@
       <c r="H86" t="b">
         <v>1</v>
       </c>
+      <c r="I86" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -9044,6 +10019,9 @@
       <c r="H87" t="b">
         <v>1</v>
       </c>
+      <c r="I87" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -9072,6 +10050,9 @@
       <c r="H88" t="b">
         <v>1</v>
       </c>
+      <c r="I88" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -9100,6 +10081,9 @@
       <c r="H89" t="b">
         <v>1</v>
       </c>
+      <c r="I89" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -9128,6 +10112,9 @@
       <c r="H90" t="b">
         <v>1</v>
       </c>
+      <c r="I90" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -9156,6 +10143,9 @@
       <c r="H91" t="b">
         <v>1</v>
       </c>
+      <c r="I91" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -9184,6 +10174,9 @@
       <c r="H92" t="b">
         <v>1</v>
       </c>
+      <c r="I92" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -9212,6 +10205,9 @@
       <c r="H93" t="b">
         <v>1</v>
       </c>
+      <c r="I93" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -9240,6 +10236,9 @@
       <c r="H94" t="b">
         <v>1</v>
       </c>
+      <c r="I94" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -9268,6 +10267,9 @@
       <c r="H95" t="b">
         <v>1</v>
       </c>
+      <c r="I95" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -9296,6 +10298,9 @@
       <c r="H96" t="b">
         <v>1</v>
       </c>
+      <c r="I96" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -9324,6 +10329,9 @@
       <c r="H97" t="b">
         <v>1</v>
       </c>
+      <c r="I97" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -9364,6 +10372,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -9396,6 +10409,9 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="I99" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -9428,6 +10444,9 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="I100" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -9460,6 +10479,9 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="I101" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -9487,6 +10509,9 @@
       </c>
       <c r="H102" t="b">
         <v>0</v>
+      </c>
+      <c r="I102" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -9500,56 +10525,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Planning</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Length</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Expected</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Missing Cases</t>
         </is>
@@ -9585,6 +10610,7 @@
           <t>✓ Done</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9688,6 +10714,7 @@
           <t>✓ Done</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9791,6 +10818,7 @@
           <t>✓ Done</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9822,6 +10850,7 @@
           <t>✓ Done</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9889,6 +10918,7 @@
           <t>✓ Done</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9920,6 +10950,7 @@
           <t>✓ Done</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9987,6 +11018,7 @@
           <t>✓ Done</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -10090,6 +11122,7 @@
           <t>✓ Done</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -10193,6 +11226,7 @@
           <t>✓ Done</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -10224,6 +11258,7 @@
           <t>✓ Done</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -10258,6 +11293,110 @@
       <c r="H22" t="inlineStr">
         <is>
           <t>[96, 97, 98, 99]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Operator-driven</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>100</v>
+      </c>
+      <c r="E23" t="n">
+        <v>100</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>✓ Done</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Operator-driven</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>85</v>
+      </c>
+      <c r="E24" t="n">
+        <v>81</v>
+      </c>
+      <c r="F24" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>⚠ Partial</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>[62, 63, 64, 87]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Operator-driven</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>L9</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>101</v>
+      </c>
+      <c r="E25" t="n">
+        <v>84</v>
+      </c>
+      <c r="F25" t="n">
+        <v>17</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>⚠ Partial</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>[13, 18, 20, 21, 36, 41, 42, 43, 44, 45, 62, 71, 72, 74, 78, 79, 96]</t>
         </is>
       </c>
     </row>
@@ -10272,38 +11411,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Planning</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Length</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Source CSV</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Exists</t>
         </is>
@@ -10327,7 +11466,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_1_rerun_without_materialization_0_100_20260305_013029/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_1_rerun_without_materialization_0_100_20260305_013029/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E2" t="b">
@@ -10352,7 +11491,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_15_48_20260305_123232/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_15_48_20260305_123232/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E3" t="b">
@@ -10377,7 +11516,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_34_67_20260305_123137/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_34_67_20260305_123137/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E4" t="b">
@@ -10402,7 +11541,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_48_81_20260305_123238/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_48_81_20260305_123238/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E5" t="b">
@@ -10427,7 +11566,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_81_100_20260305_123252/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_81_100_20260305_123252/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E6" t="b">
@@ -10452,7 +11591,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/overnight_ms_l9_0_50_20260309_012433/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/overnight_ms_l9_0_50_20260309_012433/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E7" t="b">
@@ -10477,7 +11616,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/overnight_ms_l9_51_100_20260309_012433/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/overnight_ms_l9_51_100_20260309_012433/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E8" t="b">
@@ -10502,7 +11641,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/l9_run2_ms_74_100_20260309_184346/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/l9_run2_ms_74_100_20260309_184346/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E9" t="b">
@@ -10527,7 +11666,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_1_rerun_without_materialization_0_100_20260305_013029/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_1_rerun_without_materialization_0_100_20260305_013029/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E10" t="b">
@@ -10552,7 +11691,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_15_48_20260305_123232/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_15_48_20260305_123232/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E11" t="b">
@@ -10577,7 +11716,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_34_67_20260305_123137/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_34_67_20260305_123137/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E12" t="b">
@@ -10602,7 +11741,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_48_81_20260305_123238/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_48_81_20260305_123238/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E13" t="b">
@@ -10627,7 +11766,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_81_100_20260305_123252/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/len_4_rerun_without_materialization_81_100_20260305_123252/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E14" t="b">
@@ -10652,7 +11791,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/overnight_ms_l9_0_50_20260309_012433/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/overnight_ms_l9_0_50_20260309_012433/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E15" t="b">
@@ -10677,7 +11816,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/overnight_ms_l9_51_100_20260309_012433/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/overnight_ms_l9_51_100_20260309_012433/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E16" t="b">
@@ -10702,7 +11841,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/l9_run2_ms_74_100_20260309_184346/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/l9_run2_ms_74_100_20260309_184346/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E17" t="b">
@@ -10727,7 +11866,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/AgentFlow/results/l1_run1_af_op_0_49_20260310_112706/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/AgentFlow/results/l1_run1_af_op_0_49_20260310_112706/results_summary.csv</t>
         </is>
       </c>
       <c r="E18" t="b">
@@ -10752,7 +11891,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/AgentFlow/results/l1_run1_af_op_50_99_20260310_112706/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/AgentFlow/results/l1_run1_af_op_50_99_20260310_112706/results_summary.csv</t>
         </is>
       </c>
       <c r="E19" t="b">
@@ -10777,7 +11916,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/AgentFlow/results/agentflow_operator_l1_90_100_20260310_234024/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/AgentFlow/results/agentflow_operator_l1_90_100_20260310_234024/results_summary.csv</t>
         </is>
       </c>
       <c r="E20" t="b">
@@ -10802,7 +11941,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/AgentFlow/results/l4_run1_af_op_15_57_20260310_001841/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/AgentFlow/results/l4_run1_af_op_15_57_20260310_001841/results_summary.csv</t>
         </is>
       </c>
       <c r="E21" t="b">
@@ -10827,7 +11966,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/AgentFlow/results/l4_run1_af_op_58_99_20260310_001840/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/AgentFlow/results/l4_run1_af_op_58_99_20260310_001840/results_summary.csv</t>
         </is>
       </c>
       <c r="E22" t="b">
@@ -10852,7 +11991,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/AgentFlow/results/l9_run2_af_op_0_50_20260309_190123/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/AgentFlow/results/l9_run2_af_op_0_50_20260309_190123/results_summary.csv</t>
         </is>
       </c>
       <c r="E23" t="b">
@@ -10877,7 +12016,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/AgentFlow/results/l9_run2_af_op_51_100_20260309_190123/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/AgentFlow/results/l9_run2_af_op_51_100_20260309_190123/results_summary.csv</t>
         </is>
       </c>
       <c r="E24" t="b">
@@ -10902,7 +12041,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/Langraph/results_langraph/l4_run1_mcts_15_57_20260310_062719/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/Langraph/results_langraph/l4_run1_mcts_15_57_20260310_062719/results_summary.csv</t>
         </is>
       </c>
       <c r="E25" t="b">
@@ -10927,7 +12066,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/Langraph/results_langraph/l4_run1_mcts_58_99_20260310_062719/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/Langraph/results_langraph/l4_run1_mcts_58_99_20260310_062719/results_summary.csv</t>
         </is>
       </c>
       <c r="E26" t="b">
@@ -10952,7 +12091,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/Langraph/results_langraph/l9_run2_mcts_0_50_20260310_081151/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/Langraph/results_langraph/l9_run2_mcts_0_50_20260310_081151/results_summary.csv</t>
         </is>
       </c>
       <c r="E27" t="b">
@@ -10977,7 +12116,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/Langraph/results_langraph/l9_run2_mcts_51_100_20260310_081151/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/Langraph/results_langraph/l9_run2_mcts_51_100_20260310_081151/results_summary.csv</t>
         </is>
       </c>
       <c r="E28" t="b">
@@ -11002,7 +12141,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/l1_run1_sscot_0_99_20260310_100327/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/l1_run1_sscot_0_99_20260310_100327/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E29" t="b">
@@ -11027,7 +12166,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/l4_run1_sscot_15_99_20260310_100327/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/l4_run1_sscot_15_99_20260310_100327/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E30" t="b">
@@ -11052,7 +12191,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/l9_run1_sscot_0_100_20260310_100327/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/l9_run1_sscot_0_100_20260310_100327/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E31" t="b">
@@ -11077,7 +12216,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/l1_run1_sscot_0_99_20260310_100327/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/l1_run1_sscot_0_99_20260310_100327/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E32" t="b">
@@ -11102,7 +12241,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/l4_run1_sscot_15_99_20260310_100327/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/l4_run1_sscot_15_99_20260310_100327/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E33" t="b">
@@ -11127,7 +12266,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/logs-auto-suggest-llm-21-04/l9_run1_sscot_0_100_20260310_100327/results/multi_step.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/l9_run1_sscot_0_100_20260310_100327/results/multi_step.csv</t>
         </is>
       </c>
       <c r="E34" t="b">
@@ -11152,7 +12291,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/AgentFlow/results/agentflow_pipeline_l1_20260310_234018/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/AgentFlow/results/agentflow_pipeline_l1_20260310_234018/results_summary.csv</t>
         </is>
       </c>
       <c r="E35" t="b">
@@ -11177,7 +12316,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/AgentFlow/results/l4_run1_af_pl_15_57_20260310_034423/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/AgentFlow/results/l4_run1_af_pl_15_57_20260310_034423/results_summary.csv</t>
         </is>
       </c>
       <c r="E36" t="b">
@@ -11202,7 +12341,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/AgentFlow/results/l4_run1_af_pl_58_99_20260310_034423/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/AgentFlow/results/l4_run1_af_pl_58_99_20260310_034423/results_summary.csv</t>
         </is>
       </c>
       <c r="E37" t="b">
@@ -11227,7 +12366,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/AgentFlow/results/l9_run2_af_pl_0_50_20260310_000446/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/AgentFlow/results/l9_run2_af_pl_0_50_20260310_000446/results_summary.csv</t>
         </is>
       </c>
       <c r="E38" t="b">
@@ -11252,10 +12391,160 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>/home/local/ASUAD/jrtandel/transchema/AgentFlow/results/l9_run2_af_pl_51_100_20260310_000446/results_summary.csv</t>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/AgentFlow/results/l9_run2_af_pl_51_100_20260310_000446/results_summary.csv</t>
         </is>
       </c>
       <c r="E39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Operator-driven</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/l1_4.1mini_ms_mat_0_49_20260316_215021/results/multi_step.csv</t>
+        </is>
+      </c>
+      <c r="E40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Operator-driven</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/l1_4.1mini_ms_mat_50_99_20260316_215021/results/multi_step.csv</t>
+        </is>
+      </c>
+      <c r="E41" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Operator-driven</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/l4_4.1mini_ms_mat_15_56_20260316_231146/results/multi_step.csv</t>
+        </is>
+      </c>
+      <c r="E42" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Operator-driven</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/l4_4.1mini_ms_mat_57_99_20260316_231146/results/multi_step.csv</t>
+        </is>
+      </c>
+      <c r="E43" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Operator-driven</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>L9</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/l9_4.1mini_ms_mat_0_50_20260317_021700/results/multi_step.csv</t>
+        </is>
+      </c>
+      <c r="E44" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Operator-driven</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Critique+Mat (4.1-mini)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>L9</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>/home/asurite.ad.asu.edu/jrtandel/transchema/logs-auto-suggest-llm-21-04/l9_4.1mini_ms_mat_51_100_20260317_021700/results/multi_step.csv</t>
+        </is>
+      </c>
+      <c r="E45" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>